<commit_message>
Restructure analysis pipeline into numbered scripts; consolidate old scripts
Flattens scripts/glm_analysis/ into scripts/ as a numbered pipeline
(1_loading_cleaning.R through 5_results_report.qmd) with a run_all.R
entry point and a dedicated intermediate_outputs/ folder for regenerable
.RData files. Also fixes a broken source() path left over from an
in-progress rename, and consolidates old_analyses_and_misc_scripts/ into
misc/.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/2023/thickOb_140823.xlsx
+++ b/data/raw/2023/thickOb_140823.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lunduniversityo365-my.sharepoint.com/personal/an4718sc_lu_se/Documents/PhD/projects/dorsal_snapshot_discrimination_project/analysis/data/raw/2023/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57FEC3AC-6CAA-6447-A981-D22901ABA0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{57FEC3AC-6CAA-6447-A981-D22901ABA0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A05B2740-6792-7A4A-93B6-459A44DA3D41}"/>
   <bookViews>
-    <workbookView xWindow="7260" yWindow="3520" windowWidth="27240" windowHeight="16440" activeTab="1" xr2:uid="{AF145AF8-E192-E042-85CD-F204A5937D94}"/>
+    <workbookView xWindow="7260" yWindow="3520" windowWidth="27240" windowHeight="16440" xr2:uid="{AF145AF8-E192-E042-85CD-F204A5937D94}"/>
   </bookViews>
   <sheets>
     <sheet name="thickOb_140823" sheetId="2" r:id="rId1"/>
@@ -40,195 +40,194 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="62">
   <si>
+    <t>illegible_handwriting</t>
+  </si>
+  <si>
+    <t>unmarked_ind</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>0,0,1</t>
+  </si>
+  <si>
+    <t>0,0,0,B</t>
+  </si>
+  <si>
+    <t>0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,1</t>
+  </si>
+  <si>
+    <t>1,1</t>
+  </si>
+  <si>
+    <t>0,0,0,0,B</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,1</t>
+  </si>
+  <si>
+    <t>0,0,B</t>
+  </si>
+  <si>
+    <t>36R</t>
+  </si>
+  <si>
+    <t>35L</t>
+  </si>
+  <si>
+    <t>34L</t>
+  </si>
+  <si>
+    <t>33R</t>
+  </si>
+  <si>
+    <t>32L</t>
+  </si>
+  <si>
+    <t>31L</t>
+  </si>
+  <si>
+    <t>30L</t>
+  </si>
+  <si>
+    <t>29R</t>
+  </si>
+  <si>
+    <t>28L</t>
+  </si>
+  <si>
+    <t>27R</t>
+  </si>
+  <si>
+    <t>26L</t>
+  </si>
+  <si>
+    <t>25R</t>
+  </si>
+  <si>
+    <t>24L</t>
+  </si>
+  <si>
+    <t>23R</t>
+  </si>
+  <si>
+    <t>22L</t>
+  </si>
+  <si>
+    <t>21R</t>
+  </si>
+  <si>
+    <t>20R</t>
+  </si>
+  <si>
+    <t>19L</t>
+  </si>
+  <si>
+    <t>18R</t>
+  </si>
+  <si>
+    <t>17L</t>
+  </si>
+  <si>
+    <t>16R</t>
+  </si>
+  <si>
+    <t>15L</t>
+  </si>
+  <si>
+    <t>14R</t>
+  </si>
+  <si>
+    <t>13R</t>
+  </si>
+  <si>
+    <t>12L</t>
+  </si>
+  <si>
+    <t>11L</t>
+  </si>
+  <si>
+    <t>10R</t>
+  </si>
+  <si>
+    <t>9L</t>
+  </si>
+  <si>
+    <t>7R</t>
+  </si>
+  <si>
+    <t>6R</t>
+  </si>
+  <si>
+    <t>5L</t>
+  </si>
+  <si>
+    <t>4R</t>
+  </si>
+  <si>
+    <t>3L</t>
+  </si>
+  <si>
+    <t>2L</t>
+  </si>
+  <si>
+    <t>1R</t>
+  </si>
+  <si>
+    <t>individual</t>
+  </si>
+  <si>
+    <t>1,0</t>
+  </si>
+  <si>
+    <t>48R</t>
+  </si>
+  <si>
+    <t>47R</t>
+  </si>
+  <si>
+    <t>46L</t>
+  </si>
+  <si>
+    <t>45L</t>
+  </si>
+  <si>
+    <t>44R</t>
+  </si>
+  <si>
+    <t>43R</t>
+  </si>
+  <si>
+    <t>42L</t>
+  </si>
+  <si>
+    <t>41R</t>
+  </si>
+  <si>
+    <t>40R</t>
+  </si>
+  <si>
+    <t>39R</t>
+  </si>
+  <si>
+    <t>38R</t>
+  </si>
+  <si>
+    <t>37L</t>
+  </si>
+  <si>
     <t xml:space="preserve">notes:
-This exp run over two days, need to split the excel sheet into two by day
 trial length: I see from my notes as well that trials were 4 minutes instead of the 5 I've done in later experiments. This could easily explain differences in learning rates seen in figures right?
 What was the orientation of the two stripes? I can't find this in my notes
 Perhaps it's safe to assume that rewarding stripes were from right to left (moving from front to back of maze) because this is whsat i did for the thin oblique stripes
 </t>
-  </si>
-  <si>
-    <t>illegible_handwriting</t>
-  </si>
-  <si>
-    <t>unmarked_ind</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>0,0,1</t>
-  </si>
-  <si>
-    <t>0,0,0,B</t>
-  </si>
-  <si>
-    <t>0,0,0</t>
-  </si>
-  <si>
-    <t>0,0,0,1</t>
-  </si>
-  <si>
-    <t>1,1</t>
-  </si>
-  <si>
-    <t>0,0,0,0,B</t>
-  </si>
-  <si>
-    <t>0,0,0,0,0,0</t>
-  </si>
-  <si>
-    <t>0,0,0,0,1</t>
-  </si>
-  <si>
-    <t>0,0,B</t>
-  </si>
-  <si>
-    <t>36R</t>
-  </si>
-  <si>
-    <t>35L</t>
-  </si>
-  <si>
-    <t>34L</t>
-  </si>
-  <si>
-    <t>33R</t>
-  </si>
-  <si>
-    <t>32L</t>
-  </si>
-  <si>
-    <t>31L</t>
-  </si>
-  <si>
-    <t>30L</t>
-  </si>
-  <si>
-    <t>29R</t>
-  </si>
-  <si>
-    <t>28L</t>
-  </si>
-  <si>
-    <t>27R</t>
-  </si>
-  <si>
-    <t>26L</t>
-  </si>
-  <si>
-    <t>25R</t>
-  </si>
-  <si>
-    <t>24L</t>
-  </si>
-  <si>
-    <t>23R</t>
-  </si>
-  <si>
-    <t>22L</t>
-  </si>
-  <si>
-    <t>21R</t>
-  </si>
-  <si>
-    <t>20R</t>
-  </si>
-  <si>
-    <t>19L</t>
-  </si>
-  <si>
-    <t>18R</t>
-  </si>
-  <si>
-    <t>17L</t>
-  </si>
-  <si>
-    <t>16R</t>
-  </si>
-  <si>
-    <t>15L</t>
-  </si>
-  <si>
-    <t>14R</t>
-  </si>
-  <si>
-    <t>13R</t>
-  </si>
-  <si>
-    <t>12L</t>
-  </si>
-  <si>
-    <t>11L</t>
-  </si>
-  <si>
-    <t>10R</t>
-  </si>
-  <si>
-    <t>9L</t>
-  </si>
-  <si>
-    <t>7R</t>
-  </si>
-  <si>
-    <t>6R</t>
-  </si>
-  <si>
-    <t>5L</t>
-  </si>
-  <si>
-    <t>4R</t>
-  </si>
-  <si>
-    <t>3L</t>
-  </si>
-  <si>
-    <t>2L</t>
-  </si>
-  <si>
-    <t>1R</t>
-  </si>
-  <si>
-    <t>individual</t>
-  </si>
-  <si>
-    <t>1,0</t>
-  </si>
-  <si>
-    <t>48R</t>
-  </si>
-  <si>
-    <t>47R</t>
-  </si>
-  <si>
-    <t>46L</t>
-  </si>
-  <si>
-    <t>45L</t>
-  </si>
-  <si>
-    <t>44R</t>
-  </si>
-  <si>
-    <t>43R</t>
-  </si>
-  <si>
-    <t>42L</t>
-  </si>
-  <si>
-    <t>41R</t>
-  </si>
-  <si>
-    <t>40R</t>
-  </si>
-  <si>
-    <t>39R</t>
-  </si>
-  <si>
-    <t>38R</t>
-  </si>
-  <si>
-    <t>37L</t>
   </si>
 </sst>
 </file>
@@ -620,112 +619,112 @@
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="R1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="T1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="U1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="V1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="W1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="X1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Y1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Z1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AA1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AB1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AC1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AD1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AE1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AF1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AG1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AH1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AI1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AJ1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.2">
@@ -820,10 +819,10 @@
         <v>1</v>
       </c>
       <c r="AH2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ2">
         <v>1</v>
@@ -855,13 +854,13 @@
         <v>1</v>
       </c>
       <c r="V3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="W3">
         <v>1</v>
       </c>
       <c r="X3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Y3">
         <v>1</v>
@@ -882,7 +881,7 @@
         <v>1</v>
       </c>
       <c r="AE3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF3">
         <v>1</v>
@@ -897,7 +896,7 @@
         <v>1</v>
       </c>
       <c r="AJ3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.2">
@@ -914,7 +913,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -926,16 +925,16 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O4">
         <v>1</v>
       </c>
       <c r="P4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q4">
         <v>1</v>
@@ -950,7 +949,7 @@
         <v>0</v>
       </c>
       <c r="U4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V4">
         <v>1</v>
@@ -1038,85 +1037,85 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
         <v>3</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="I6" t="s">
-        <v>4</v>
-      </c>
       <c r="J6">
         <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L6" t="s">
+        <v>6</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" t="s">
         <v>7</v>
       </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>1</v>
-      </c>
-      <c r="O6" t="s">
-        <v>4</v>
-      </c>
-      <c r="P6" t="s">
-        <v>8</v>
-      </c>
       <c r="Q6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R6">
         <v>1</v>
       </c>
       <c r="S6" t="s">
+        <v>2</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>1</v>
+      </c>
+      <c r="V6" t="s">
+        <v>2</v>
+      </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6">
+        <v>1</v>
+      </c>
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA6">
+        <v>1</v>
+      </c>
+      <c r="AB6">
+        <v>1</v>
+      </c>
+      <c r="AC6">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>2</v>
+      </c>
+      <c r="AF6" t="s">
         <v>3</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <v>1</v>
-      </c>
-      <c r="V6" t="s">
-        <v>3</v>
-      </c>
-      <c r="W6">
-        <v>1</v>
-      </c>
-      <c r="X6">
-        <v>1</v>
-      </c>
-      <c r="Y6">
-        <v>1</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA6">
-        <v>1</v>
-      </c>
-      <c r="AB6">
-        <v>1</v>
-      </c>
-      <c r="AC6">
-        <v>1</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF6" t="s">
-        <v>4</v>
       </c>
       <c r="AG6">
         <v>1</v>
@@ -1145,53 +1144,53 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H7" t="s">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>1</v>
+      </c>
+      <c r="R7" t="s">
+        <v>2</v>
+      </c>
+      <c r="S7" t="s">
+        <v>2</v>
+      </c>
+      <c r="U7" t="s">
         <v>3</v>
       </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="J7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
-      <c r="O7">
-        <v>1</v>
-      </c>
-      <c r="P7">
-        <v>1</v>
-      </c>
-      <c r="Q7">
-        <v>1</v>
-      </c>
-      <c r="R7" t="s">
-        <v>3</v>
-      </c>
-      <c r="S7" t="s">
-        <v>3</v>
-      </c>
-      <c r="U7" t="s">
-        <v>4</v>
-      </c>
       <c r="V7">
         <v>1</v>
       </c>
@@ -1202,13 +1201,13 @@
         <v>1</v>
       </c>
       <c r="Y7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z7">
         <v>1</v>
       </c>
       <c r="AA7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB7">
         <v>1</v>
@@ -1240,12 +1239,12 @@
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -1253,7 +1252,7 @@
     </row>
     <row r="12" spans="1:36" ht="409.6" x14ac:dyDescent="0.2">
       <c r="B12" s="2" t="s">
-        <v>0</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1272,43 +1271,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="M1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
@@ -1322,7 +1321,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1340,10 +1339,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -1374,13 +1373,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1436,7 +1435,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -1468,7 +1467,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -1477,7 +1476,7 @@
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -1491,25 +1490,25 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
         <v>3</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>4</v>
-      </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -1526,12 +1525,12 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>